<commit_message>
Updated preconfig-advanced.xlsx with EdgeHA information.
</commit_message>
<xml_diff>
--- a/examples/generate_preconfig/preconfig-advanced.xlsx
+++ b/examples/generate_preconfig/preconfig-advanced.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilkinad\OneDrive - Hewlett Packard Enterprise\Documents\PycharmProjects\Pyedgeconnect_Dev\pyedgeconnect\examples\generate_preconfig\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpe-my.sharepoint.com/personal/adam_wilkins_hpe_com/Documents/Documents/PycharmProjects/Pyedgeconnect_Dev/pyedgeconnect/examples/generate_preconfig/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AB9E752-221B-4615-A8C1-F2FDFF1D0BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{6AB9E752-221B-4615-A8C1-F2FDFF1D0BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2B8E10D-397B-421C-9029-8FCA41E1E75B}"/>
   <bookViews>
-    <workbookView xWindow="6160" yWindow="3180" windowWidth="28800" windowHeight="11250" xr2:uid="{7F121074-DE26-455A-91EF-616A72B8B77B}"/>
+    <workbookView xWindow="7790" yWindow="4030" windowWidth="28800" windowHeight="11250" xr2:uid="{7F121074-DE26-455A-91EF-616A72B8B77B}"/>
   </bookViews>
   <sheets>
     <sheet name="preconfig-advanced" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="187">
   <si>
     <t>softwareVersion</t>
   </si>
@@ -485,6 +485,102 @@
   </si>
   <si>
     <t>Unlimited</t>
+  </si>
+  <si>
+    <t>haPeerSerial</t>
+  </si>
+  <si>
+    <t>haPeerHostname</t>
+  </si>
+  <si>
+    <t>haIPPool</t>
+  </si>
+  <si>
+    <t>haSubnetMask</t>
+  </si>
+  <si>
+    <t>haVlanStart</t>
+  </si>
+  <si>
+    <t>haInterface</t>
+  </si>
+  <si>
+    <t>haInterfaceOrder</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel1</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel1_outboundbw</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel1_inboundbw</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel1_segment</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel1_zone</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel2</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel2_outboundbw</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel2_inboundbw</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel2_segment</t>
+  </si>
+  <si>
+    <t>haPeerInterfaceInfo_interfaceLabel2_zone</t>
+  </si>
+  <si>
+    <t>EdgeHA1</t>
+  </si>
+  <si>
+    <t>EdgeHA2</t>
+  </si>
+  <si>
+    <t>Frisco</t>
+  </si>
+  <si>
+    <t>wan2</t>
+  </si>
+  <si>
+    <t>MPLS1, INET1, INET2</t>
+  </si>
+  <si>
+    <t>MPLS1</t>
+  </si>
+  <si>
+    <t>172.23.14.2/24</t>
+  </si>
+  <si>
+    <t>172.23.14.3/24</t>
+  </si>
+  <si>
+    <t>151.85.33.50/29</t>
+  </si>
+  <si>
+    <t>151.85.33.49</t>
+  </si>
+  <si>
+    <t>12.33.2.66/30</t>
+  </si>
+  <si>
+    <t>12.33.2.65/30</t>
+  </si>
+  <si>
+    <t>MPLS</t>
+  </si>
+  <si>
+    <t>23.85.33.130/29</t>
+  </si>
+  <si>
+    <t>23.85.33.129</t>
   </si>
 </sst>
 </file>
@@ -627,7 +723,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -807,8 +903,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -923,6 +1025,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -968,8 +1085,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1026,6 +1144,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1345,277 +1467,331 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD26F203-BEC6-4B24-88A3-71D204A42B80}">
-  <dimension ref="A1:CJ5"/>
+  <dimension ref="A1:DA7"/>
   <sheetFormatPr defaultColWidth="33.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="70" max="78" width="44.90625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:88" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:105" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BJ1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="BV1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="BW1" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="BX1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="BY1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="CA1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="CB1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="CC1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="CE1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="CF1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="CG1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="CH1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="CI1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CJ1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CK1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CL1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CM1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CN1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CO1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CP1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CQ1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CR1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CT1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CU1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CV1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CW1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CX1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CY1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CZ1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="DA1" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:88" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
+    <row r="2" spans="1:105" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>88</v>
       </c>
       <c r="C2" t="s">
@@ -1714,18 +1890,18 @@
       <c r="BH2" t="s">
         <v>109</v>
       </c>
-      <c r="BV2">
+      <c r="CL2">
         <v>100000</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CX2" t="s">
         <v>115</v>
       </c>
-      <c r="CI2" t="s">
+      <c r="CY2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:88" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+    <row r="3" spans="1:105" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>117</v>
       </c>
       <c r="C3" t="s">
@@ -1824,18 +2000,18 @@
       <c r="BH3" t="s">
         <v>109</v>
       </c>
-      <c r="BV3">
+      <c r="CL3">
         <v>100000</v>
       </c>
-      <c r="CH3" t="s">
+      <c r="CX3" t="s">
         <v>115</v>
       </c>
-      <c r="CI3" t="s">
+      <c r="CY3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:88" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    <row r="4" spans="1:105" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>129</v>
       </c>
       <c r="C4" t="s">
@@ -1934,18 +2110,18 @@
       <c r="BH4" t="s">
         <v>109</v>
       </c>
-      <c r="BV4">
+      <c r="CL4">
         <v>100000</v>
       </c>
-      <c r="CH4" t="s">
+      <c r="CX4" t="s">
         <v>115</v>
       </c>
-      <c r="CI4" t="s">
+      <c r="CY4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:88" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+    <row r="5" spans="1:105" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>141</v>
       </c>
       <c r="E5" t="s">
@@ -2029,11 +2205,208 @@
       <c r="BH5" t="s">
         <v>109</v>
       </c>
-      <c r="BU5" t="s">
+      <c r="CK5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:105" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6" t="s">
+        <v>174</v>
+      </c>
+      <c r="G6" t="s">
+        <v>143</v>
+      </c>
+      <c r="J6" t="s">
+        <v>174</v>
+      </c>
+      <c r="K6" t="s">
+        <v>92</v>
+      </c>
+      <c r="S6" t="s">
+        <v>93</v>
+      </c>
+      <c r="T6" t="s">
+        <v>94</v>
+      </c>
+      <c r="U6">
+        <v>100000</v>
+      </c>
+      <c r="V6">
+        <v>300000</v>
+      </c>
+      <c r="W6">
+        <v>100000</v>
+      </c>
+      <c r="X6">
+        <v>300000</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>145</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>178</v>
+      </c>
+      <c r="AT6" t="s">
+        <v>104</v>
+      </c>
+      <c r="AU6" t="s">
+        <v>148</v>
+      </c>
+      <c r="AV6" t="s">
+        <v>105</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>180</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>181</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>108</v>
+      </c>
+      <c r="AZ6" t="s">
+        <v>109</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>110</v>
+      </c>
+      <c r="BC6" t="s">
+        <v>184</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>177</v>
+      </c>
+      <c r="BE6" t="s">
+        <v>185</v>
+      </c>
+      <c r="BF6" t="s">
+        <v>186</v>
+      </c>
+      <c r="BG6" t="s">
+        <v>108</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>109</v>
+      </c>
+      <c r="BK6" t="s">
+        <v>173</v>
+      </c>
+      <c r="BO6" t="s">
+        <v>175</v>
+      </c>
+      <c r="BP6" t="s">
+        <v>176</v>
+      </c>
+      <c r="BQ6" t="s">
+        <v>112</v>
+      </c>
+      <c r="BR6">
+        <v>80000</v>
+      </c>
+      <c r="BS6">
+        <v>80000</v>
+      </c>
+      <c r="CK6" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:105" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E7" t="s">
+        <v>174</v>
+      </c>
+      <c r="G7" t="s">
+        <v>143</v>
+      </c>
+      <c r="J7" t="s">
+        <v>174</v>
+      </c>
+      <c r="K7" t="s">
+        <v>92</v>
+      </c>
+      <c r="S7" t="s">
+        <v>93</v>
+      </c>
+      <c r="T7" t="s">
+        <v>94</v>
+      </c>
+      <c r="U7">
+        <v>80000</v>
+      </c>
+      <c r="W7">
+        <v>80000</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>145</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>179</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>104</v>
+      </c>
+      <c r="AU7" t="s">
+        <v>148</v>
+      </c>
+      <c r="AV7" t="s">
+        <v>112</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>182</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>183</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>108</v>
+      </c>
+      <c r="AZ7" t="s">
+        <v>109</v>
+      </c>
+      <c r="BK7" t="s">
+        <v>172</v>
+      </c>
+      <c r="BO7" t="s">
+        <v>175</v>
+      </c>
+      <c r="BP7" t="s">
+        <v>176</v>
+      </c>
+      <c r="BQ7" t="s">
+        <v>105</v>
+      </c>
+      <c r="BR7">
+        <v>100000</v>
+      </c>
+      <c r="BS7">
+        <v>100000</v>
+      </c>
+      <c r="BV7" t="s">
+        <v>177</v>
+      </c>
+      <c r="BW7">
+        <v>300000</v>
+      </c>
+      <c r="BX7">
+        <v>300000</v>
+      </c>
+      <c r="CK7" t="s">
         <v>154</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>